<commit_message>
Update petit-traitor gallery spreadsheet (43 rows)
</commit_message>
<xml_diff>
--- a/petit-traitor-gallery.xlsx
+++ b/petit-traitor-gallery.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1258,6 +1258,23 @@
       <c r="D43" s="5" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr"/>
     </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>photo-20260828-062303.jpg</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260828-062303.jpg</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update gallery spreadsheet with clickable photo links
</commit_message>
<xml_diff>
--- a/petit-traitor-gallery.xlsx
+++ b/petit-traitor-gallery.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,12 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="5">
@@ -77,19 +83,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -464,7 +482,7 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
@@ -482,7 +500,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Thumbnail URL</t>
+          <t>View Photo (click)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -500,782 +518,826 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-023604.jpg</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-023604.jpg</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Tell him not to wait. Your day's been planned by hands that don't belong to him.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>photo-20260707-185745-02.jpg</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260707-185745-02.jpg</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Escaping on a vessel while hubby is home,  just met the captain.</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>photo-20260823-064054.jpg</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-064054.jpg</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>He thinks I'm off to find some spiritual clarity at the harbor by myself. He doesn't know I'm off to meet a tall, rich 64-year-old man who actually listens to me. He understands my soul.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>photo-20260823-064715.jpg</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-064715.jpg</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Not her husband</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>photo-20260823-064717-01.jpg</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-064717-01.jpg</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Not her husband</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>photo-20260823-064720-02.jpg</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-064720-02.jpg</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Not her husband</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>photo-20260823-203905.jpg</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-203905.jpg</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>On a quiet ferry ride, the Filipino fiancée leans into her secret lover—the older American man who's been spoiling her since she arrived. Her K-1 fiancé has no idea she's already giving her heart (and body) to someone else while he waits back home processing the paperwork.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>photo-20260823-203907-01.jpg</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-203907-01.jpg</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>photo-20260823-203910-02.jpg</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-203910-02.jpg</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>She rises on her toes and claims his mouth like she owns it, and will press her barely-covered tits against his chest. The same lips that promised forever to her American sponsor are now hungry for the man who's been fucking her raw on this trip.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>photo-20260823-203912-03.jpg</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-203912-03.jpg</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>photo-20260823-203915-04.jpg</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-203915-04.jpg</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Caught red-handed. Her fiancé stands there stunned while she stays half-naked between the two men, still glowing from the older guy's touch. The lover shrugs like it's no big deal that he's been deep inside the woman the younger man was about to marry.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>photo-20260823-203917-05.jpg</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260823-203917-05.jpg</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>She doesn't even flinch. Instead she plants her hands on her fiancé's chest and shoves him back, choosing the older man who's been bending her over every chance he gets over the one who was ready to give her a green card and a wedding.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-133801.jpg</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-133801.jpg</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>She tamed them not with words, but with the slow, deliberate rhythm of her body.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>photo-20260824-132235.jpg</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-132235.jpg</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-132237-01.jpg</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-132237-01.jpg</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>photo-20260824-132240-02.jpg</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-132240-02.jpg</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr"/>
+      <c r="E17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-132242-03.jpg</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-132242-03.jpg</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>photo-20260824-132245-04.jpg</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-132245-04.jpg</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr"/>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr"/>
+      <c r="E19" s="7" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-132247-05.jpg</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-132247-05.jpg</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>photo-20260824-061846.jpg</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-061846.jpg</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr"/>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr"/>
+      <c r="E21" s="7" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-061849-01.jpg</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-061849-01.jpg</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>photo-20260824-061851-02.jpg</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-061851-02.jpg</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr"/>
+      <c r="E23" s="7" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-061853-03.jpg</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-061853-03.jpg</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>photo-20260824-061856-04.jpg</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-061856-04.jpg</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr"/>
+      <c r="E25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>photo-20260824-061858-05.jpg</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260824-061858-05.jpg</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>photo-20260825-174536.jpg</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260825-174536.jpg</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr"/>
+      <c r="E27" s="7" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>photo-20260825-174538-01.jpg</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260825-174538-01.jpg</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>photo-20260825-220731.jpg</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260825-220731.jpg</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr"/>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr"/>
+      <c r="E29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>photo-20260825-220736-01.jpg</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260825-220736-01.jpg</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>photo-20260826-021354.jpg</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-021354.jpg</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>Tell Hubby not to wait. Your day has already been planned.</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr"/>
+      <c r="E31" s="7" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-070456.jpg</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070456.jpg</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>photo-20260826-070459-01.jpg</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070459-01.jpg</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr"/>
+      <c r="E33" s="7" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-070501-02.jpg</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070501-02.jpg</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>photo-20260826-070504-03.jpg</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070504-03.jpg</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr"/>
+      <c r="E35" s="7" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-070507-04.jpg</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070507-04.jpg</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>photo-20260826-070509-05.jpg</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070509-05.jpg</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr"/>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr"/>
+      <c r="E37" s="7" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-070512-06.jpg</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070512-06.jpg</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>photo-20260826-070515-07.jpg</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070515-07.jpg</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr"/>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr"/>
+      <c r="E39" s="7" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-070617.jpg</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070617.jpg</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>photo-20260826-070619-01.jpg</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070619-01.jpg</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr"/>
+      <c r="E41" s="7" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>photo-20260826-070621-02.jpg</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260826-070621-02.jpg</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="3" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="4" t="n">
+      <c r="A43" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>video-20260826-070731.mp4</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>(video — no thumbnail)</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>(video)</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr"/>
+      <c r="E43" s="7" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>photo-20260828-062303.jpg</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>https://nbiryukov25.github.io/joyce-photos-gallery/assets/Northern-Summer-Fun/photo-20260828-062303.jpg</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Open photo</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId42"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>